<commit_message>
fix(skills): reviewer pass - 44 wording fixes and the findings behind them
One independent reviewer read all ten skills top to bottom as a
smaller model would. Fixed: hand-offs between sync and interview (no
duplicate reminders or tracker notes), the thank-you shape said one
way, the guardrail block says it never covers messages or offers, the
AI-notice wording matches hard rule 7 everywhere, the six standing sync
checks, the interview quick path makes the role folder, publish has a
real secret-scan command, onboarding exports the résumé by script, a
one-page placeholder résumé in the fixture so Jane's morning routes to
sync, dates in the D Mon YYYY style in every example.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/fixtures/persona-jane-doe/hunt/job-tracker.xlsx
+++ b/assets/fixtures/persona-jane-doe/hunt/job-tracker.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Read the JD and decide by 17 Oct</t>
+          <t>You: read the JD and decide by 17 Oct</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -572,7 +572,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>14 Oct 2026: Link from a former colleague. IC role that owns the component library.</t>
+          <t>14 Oct 2026: Portfolio refresh in progress before applying || 14 Oct 2026: Link from a former colleague. IC role that owns the component library.</t>
         </is>
       </c>
     </row>

</xml_diff>